<commit_message>
Milestone 5B e-invoice.be sandbox validation
</commit_message>
<xml_diff>
--- a/test_data/workbooks/BE-VALID-001.xlsx
+++ b/test_data/workbooks/BE-VALID-001.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,70 +447,80 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>company_number</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>enterprise_number</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>legal_registration_number</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>legal_registration_scheme_id</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>address_line_1</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>address_line_2</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>postal_code</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>country_name</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>iban</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>bic</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>payment_account_name</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>peppol_id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>peppol_scheme_id</t>
         </is>
@@ -535,67 +545,77 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BE0123456789</t>
+          <t>BE0990251719</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0123456789</t>
+          <t>0990251719</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>0990251719</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0990251719</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>0208</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Rue Demo 1</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
         <is>
           <t>Brussels</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Belgium</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>billing@example.test</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>BE68539007547034</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>BBRUBEBB</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Demo Belgium Services BV</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>0208:0123456789</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>0208:0990251719</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>0208</t>
         </is>
@@ -612,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,50 +663,60 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>company_number</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>enterprise_number</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>legal_registration_number</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>legal_registration_scheme_id</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>address_line_1</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>address_line_2</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>postal_code</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>country_name</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>peppol_id</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>peppol_scheme_id</t>
         </is>
@@ -715,51 +745,61 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BE0987654321</t>
+          <t>BE0987654394</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0987654321</t>
+          <t>0987654394</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>0987654394</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0987654394</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>0208</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Buyer Street 10</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
         <is>
           <t>Antwerp</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Belgium</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>ap@example.test</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0208:0987654321</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0208:0987654394</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>0208</t>
         </is>

</xml_diff>